<commit_message>
투자 대시보드 2026-10-02 18:25
</commit_message>
<xml_diff>
--- a/technicals/exports/2026-10-01.xlsx
+++ b/technicals/exports/2026-10-01.xlsx
@@ -142,7 +142,7 @@
       </ns0:c>
       <ns0:c r="F2" t="inlineStr">
         <ns0:is>
-          <ns0:t>중국 뷰티·개인관리 브랜드에 전략, 마케팅, 전 채널 판매, 고객 서비스 및 물류 등 브랜드 관리 제공.</ns0:t>
+          <ns0:t>중국 뷰티·개인관리 브랜드에 전략·마케팅·전 채널 판매·고객 서비스·물류 등 브랜드 관리 제공.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G2">
@@ -297,7 +297,7 @@
       </ns0:c>
       <ns0:c r="F4" t="inlineStr">
         <ns0:is>
-          <ns0:t>기업·컨택센터·통신사업자에 음성 통신 인프라·장비, 클라우드 관리 및 음성 AI 솔루션 제공.</ns0:t>
+          <ns0:t>기업·컨택센터·통신사업자에 음성 통신 인프라·장비, 클라우드 관리·음성 AI 솔루션 제공.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G4">
@@ -376,7 +376,7 @@
       </ns0:c>
       <ns0:c r="F5" t="inlineStr">
         <ns0:is>
-          <ns0:t>이식 환자의 치료 결과와 장기 건강 개선을 위한 솔루션을 제공하는 기업.</ns0:t>
+          <ns0:t>이식 환자의 치료 결과와 장기 건강 개선을 위한 솔루션 제공.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G5">
@@ -455,7 +455,7 @@
       </ns0:c>
       <ns0:c r="F6" t="inlineStr">
         <ns0:is>
-          <ns0:t>기업·공공부문 등에 컴퓨터 시스템과 데이터센터를 포함한 다양한 IT 솔루션을 제공하는 기업.</ns0:t>
+          <ns0:t>기업·공공부문에 컴퓨터 시스템·데이터센터 등 다양한 IT 솔루션을 제공하는 기업.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G6">
@@ -534,7 +534,7 @@
       </ns0:c>
       <ns0:c r="F7" t="inlineStr">
         <ns0:is>
-          <ns0:t>주요 영업활동 없이 하나 이상의 기업과 합병·주식교환·자산인수 등 기업결합을 추진.</ns0:t>
+          <ns0:t>주요 영업활동 없이 하나 이상의 기업과 합병·주식교환·자산인수 등 기업결합 추진.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G7">
@@ -768,7 +768,7 @@
       </ns0:c>
       <ns0:c r="F10" t="inlineStr">
         <ns0:is>
-          <ns0:t>자회사를 통해 원유 운반선을 소유·운영하며 기술 관리 서비스도 제공하는 기업.</ns0:t>
+          <ns0:t>자회사를 통해 원유 운반선을 소유·운영하고 기술 관리 서비스 제공.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G10">
@@ -847,7 +847,7 @@
       </ns0:c>
       <ns0:c r="F11" t="inlineStr">
         <ns0:is>
-          <ns0:t>주요 영업활동 없이 기업 합병, 주식 교환, 자산 인수 등 기업결합을 추진한다.</ns0:t>
+          <ns0:t>주요 영업활동 없이 합병·주식 교환·자산 인수 등 기업결합을 추진한다.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G11">
@@ -923,7 +923,7 @@
       </ns0:c>
       <ns0:c r="F12" t="inlineStr">
         <ns0:is>
-          <ns0:t>디지털 기업의 복잡한 디지털 환경을 위한 AI 기반 관측성 플랫폼을 제공하는 기업.</ns0:t>
+          <ns0:t>기업의 복잡한 디지털 환경을 위한 AI 기반 관측성 플랫폼 제공.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G12">
@@ -1081,7 +1081,7 @@
       </ns0:c>
       <ns0:c r="F14" t="inlineStr">
         <ns0:is>
-          <ns0:t>시계·스마트워치·주얼리·핸드백·가죽 소품·벨트·선글라스 등 패션 액세서리를 설계·개발·유통.</ns0:t>
+          <ns0:t>시계·스마트워치·주얼리·핸드백·가죽 소품·벨트·선글라스 등 패션 액세서리 설계·개발·유통.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G14">
@@ -1239,7 +1239,7 @@
       </ns0:c>
       <ns0:c r="F16" t="inlineStr">
         <ns0:is>
-          <ns0:t>주요 영업활동 없이 기업 합병, 주식 교환, 자산 인수 등 기업결합을 추진한다.</ns0:t>
+          <ns0:t>주요 영업활동 없이 합병·주식 교환·자산 인수 등 기업결합을 추진한다.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G16">
@@ -1315,7 +1315,7 @@
       </ns0:c>
       <ns0:c r="F17" t="inlineStr">
         <ns0:is>
-          <ns0:t>기술로 의료 제공을 확장·자동화하며 급성 부상·만성 통증·수술 후 재활 등 근골격계 관리 플랫폼을 개발하는 기업.</ns0:t>
+          <ns0:t>급성 부상·만성 통증·수술 후 재활 등 근골격계 관리를 위한 의료 자동화 플랫폼 개발 기업.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G17">
@@ -1394,7 +1394,7 @@
       </ns0:c>
       <ns0:c r="F18" t="inlineStr">
         <ns0:is>
-          <ns0:t>미국·영국 등에서 핀테크 및 통신 솔루션을 제공하는 기업.</ns0:t>
+          <ns0:t>미국·영국 등에서 핀테크 및 통신 솔루션 제공.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G18">
@@ -1473,7 +1473,7 @@
       </ns0:c>
       <ns0:c r="F19" t="inlineStr">
         <ns0:is>
-          <ns0:t>전 세계에 전자 설계·시험용 소프트웨어, 계측기, 시스템 및 관련 서비스를 제공.</ns0:t>
+          <ns0:t>전 세계에 전자 설계·시험용 소프트웨어, 계측기·시스템 및 관련 서비스 제공.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G19">
@@ -1710,7 +1710,7 @@
       </ns0:c>
       <ns0:c r="F22" t="inlineStr">
         <ns0:is>
-          <ns0:t>보건·안전 분야에 사용하는 휴대용 질량분석기와 푸리에 변환 적외선 장비를 제공한다.</ns0:t>
+          <ns0:t>보건·안전 분야용 휴대용 질량분석기와 푸리에 변환 적외선 장비 제공.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G22">
@@ -1789,7 +1789,7 @@
       </ns0:c>
       <ns0:c r="F23" t="inlineStr">
         <ns0:is>
-          <ns0:t>자동차 금융·리스, 은행 및 금융서비스 산업용 기업 소프트웨어를 설계·개발·판매하는 회사.</ns0:t>
+          <ns0:t>자동차 금융·리스, 은행·금융서비스용 기업 소프트웨어를 설계·개발·판매하는 회사.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G23">
@@ -1947,7 +1947,7 @@
       </ns0:c>
       <ns0:c r="F25" t="inlineStr">
         <ns0:is>
-          <ns0:t>미국과 해외에서 싱글 사인온과 위험 기반 다중요소 인증 등 신원·접근 보안 서비스를 제공하는 회사.</ns0:t>
+          <ns0:t>미국과 해외에서 싱글 사인온, 위험 기반 다중요소 인증 등 신원·접근 보안 서비스를 제공하는 회사.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G25">
@@ -2026,7 +2026,7 @@
       </ns0:c>
       <ns0:c r="F26" t="inlineStr">
         <ns0:is>
-          <ns0:t>데이터 저장·관리 기술과 제품, 서비스를 제공하며 데이터 축소·보호·암호화 소프트웨어를 공급한다.</ns0:t>
+          <ns0:t>데이터 저장·관리 기술과 제품·서비스, 데이터 축소·보호·암호화 소프트웨어 제공.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G26">
@@ -2105,7 +2105,7 @@
       </ns0:c>
       <ns0:c r="F27" t="inlineStr">
         <ns0:is>
-          <ns0:t>선불카드, 환자 비용 부담 지원, 디지털뱅킹, 생명과학 소프트웨어 및 통합 결제처리를 제공하는 회사.</ns0:t>
+          <ns0:t>선불카드, 환자 비용 지원, 디지털뱅킹, 생명과학 소프트웨어 및 통합 결제처리를 제공하는 회사.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G27">
@@ -2184,7 +2184,7 @@
       </ns0:c>
       <ns0:c r="F28" t="inlineStr">
         <ns0:is>
-          <ns0:t>p53 변이 및 관련 암을 표적으로 하는 저분자 치료제를 발굴·개발하는 미국 정밀항암 기업.</ns0:t>
+          <ns0:t>p53 변이 및 관련 암을 표적으로 저분자 치료제를 발굴·개발하는 미국 정밀항암 기업.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G28">
@@ -2418,7 +2418,7 @@
       </ns0:c>
       <ns0:c r="F31" t="inlineStr">
         <ns0:is>
-          <ns0:t>기업·클라우드·SaaS 데이터 보호, 데이터 위협 분석 및 신원 복구 등 보안 솔루션을 제공하는 회사.</ns0:t>
+          <ns0:t>기업·클라우드·SaaS 데이터 보호, 데이터 위협 분석 및 신원 복구 보안 솔루션을 제공하는 회사.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G31">
@@ -2576,7 +2576,7 @@
       </ns0:c>
       <ns0:c r="F33" t="inlineStr">
         <ns0:is>
-          <ns0:t>독자 기술과 분석 역량으로 신원 정보를 제공하며, 조사 솔루션 idiCORE를 운영하는 미국 기업.</ns0:t>
+          <ns0:t>독자 기술과 분석으로 신원 정보를 제공하고 조사 솔루션 idiCORE를 운영하는 미국 기업.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G33">
@@ -2971,7 +2971,7 @@
       </ns0:c>
       <ns0:c r="F38" t="inlineStr">
         <ns0:is>
-          <ns0:t>미국과 해외에서 메시지·음성·이메일·영상 소통용 API와 소프트웨어 등 고객 참여 플랫폼을 제공한다.</ns0:t>
+          <ns0:t>미국과 해외에서 메시지·음성·이메일·영상 소통 API와 소프트웨어 등 고객 참여 플랫폼을 제공한다.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G38">
@@ -3050,7 +3050,7 @@
       </ns0:c>
       <ns0:c r="F39" t="inlineStr">
         <ns0:is>
-          <ns0:t>치료제·진단·소재·농업·데이터 저장·학술 연구 등에 쓰이는 합성 DNA 제품을 제조·판매한다.</ns0:t>
+          <ns0:t>치료제·진단·소재·농업·데이터 저장·학술 연구용 합성 DNA 제품 제조·판매.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G39">
@@ -3287,7 +3287,7 @@
       </ns0:c>
       <ns0:c r="F42" t="inlineStr">
         <ns0:is>
-          <ns0:t>유의미한 영업활동 없이 기업 합병·주식 교환·자산 인수 등 사업결합을 추진한다.</ns0:t>
+          <ns0:t>유의미한 영업활동 없이 합병·주식 교환·자산 인수 등 사업결합을 추진한다.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G42">
@@ -3363,7 +3363,7 @@
       </ns0:c>
       <ns0:c r="F43" t="inlineStr">
         <ns0:is>
-          <ns0:t>기술 서비스 분야 기업과의 합병·주식 교환·자산 인수 등 사업결합을 추진한다.</ns0:t>
+          <ns0:t>기술 서비스 기업과의 합병·주식 교환·자산 인수 등 사업결합을 추진한다.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G43">

</xml_diff>